<commit_message>
upd batch evaluation pipeline
</commit_message>
<xml_diff>
--- a/outputs/evaluation/appendix/Appendix_C_E5_Failure_Attribution.xlsx
+++ b/outputs/evaluation/appendix/Appendix_C_E5_Failure_Attribution.xlsx
@@ -49389,7 +49389,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table 4.12</t>
+          <t>Table C.1</t>
         </is>
       </c>
     </row>
@@ -49673,7 +49673,7 @@
     <row r="13" ht="104" customHeight="1">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Note. Values are the number (and percentage) of slices in each bucket. Each slice is assigned to the first failed gate, checked in the order of Section 3.4.4: X, A (head mask kept &lt; 90% of the tumor), B (&lt; 30% of the tumor in the candidate mask), C (&lt; 50% of the seed core inside the tumor), G (final DSC ≥ 0.70), F (post-processing lowered DSC by ≥ 0.10), D (growth precision &lt; 0.50 and not above recall), and E (all others). Class differences in the distribution over G, B, C, and the remaining buckets: χ²(6, N = 954) = 385.89, p &lt; .001, V = .45.</t>
+          <t>Note. Values are the number (and percentage) of slices in each bucket. Each slice is assigned to the first failed gate, checked in the order of Table 3.4: X, A (head mask kept &lt; 90% of the tumor), B (&lt; 30% of the tumor in the candidate mask), C (&lt; 50% of the seed core inside the tumor), G (final DSC ≥ 0.70), F (post-processing lowered DSC by ≥ 0.10), D (growth precision &lt; 0.50 and not above recall), and E (all others). Class differences in the distribution over G, B, C, and the remaining buckets: χ²(6, N = 954) = 385.89, p &lt; .001, V = .45.</t>
         </is>
       </c>
     </row>

</xml_diff>